<commit_message>
Add 6 more AMZ ASSET 1 main images
</commit_message>
<xml_diff>
--- a/AMZ_asset1_image_urls.xlsx
+++ b/AMZ_asset1_image_urls.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Asset 1 Packs" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Asset 1 Main'!$A$1:$D$158</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Asset 1 Main'!$A$1:$D$164</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Asset 1 Packs'!$A$1:$D$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D158"/>
+  <dimension ref="A1:D164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3928,8 +3928,140 @@
         </is>
       </c>
     </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>ML100068</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>Rick Tocchet</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>ML100068_RICK_TOCCHET_amzasset1.jpg</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="inlineStr">
+        <is>
+          <t>https://images-production-a1f5.up.railway.app/amz/asset-1/ML100068_RICK_TOCCHET_amzasset1.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>ML100105</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>William Nylander Special Edition</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>ML100105_WILLIAM_NYLANDER_SPECIAL_EDITION_amzasset1.jpg</t>
+        </is>
+      </c>
+      <c r="D160" s="3" t="inlineStr">
+        <is>
+          <t>https://images-production-a1f5.up.railway.app/amz/asset-1/ML100105_WILLIAM_NYLANDER_SPECIAL_EDITION_amzasset1.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>ML100123</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>Leon Draisaitl Home</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>ML100123_LEON_DRAISAITL_HOME_amzasset1.jpg</t>
+        </is>
+      </c>
+      <c r="D161" s="3" t="inlineStr">
+        <is>
+          <t>https://images-production-a1f5.up.railway.app/amz/asset-1/ML100123_LEON_DRAISAITL_HOME_amzasset1.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>ML100148</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>Martin Brodeur</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>ML100148_MARTIN_BRODEUR_amzasset1.jpg</t>
+        </is>
+      </c>
+      <c r="D162" s="3" t="inlineStr">
+        <is>
+          <t>https://images-production-a1f5.up.railway.app/amz/asset-1/ML100148_MARTIN_BRODEUR_amzasset1.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>ML100152</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>Sergei Fedorov</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>ML100152_SERGEI_FEDOROV_amzasset1.jpg</t>
+        </is>
+      </c>
+      <c r="D163" s="3" t="inlineStr">
+        <is>
+          <t>https://images-production-a1f5.up.railway.app/amz/asset-1/ML100152_SERGEI_FEDOROV_amzasset1.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>ML101202</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>Porter Martone</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>ML101202_PORTER_MARTONE_amzasset1.jpg</t>
+        </is>
+      </c>
+      <c r="D164" s="3" t="inlineStr">
+        <is>
+          <t>https://images-production-a1f5.up.railway.app/amz/asset-1/ML101202_PORTER_MARTONE_amzasset1.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D158"/>
+  <autoFilter ref="A1:D164"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -4088,6 +4220,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D156" r:id="rId155"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D157" r:id="rId156"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D158" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D159" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D160" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D161" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D162" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D163" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D164" r:id="rId163"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add PHL sock and package shots
</commit_message>
<xml_diff>
--- a/AMZ_asset1_image_urls.xlsx
+++ b/AMZ_asset1_image_urls.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Asset 1 Packs" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Asset 1 Main'!$A$1:$D$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Asset 1 Main'!$A$1:$D$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Asset 1 Packs'!$A$1:$D$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D164"/>
+  <dimension ref="A1:D170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4060,8 +4060,140 @@
         </is>
       </c>
     </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>ML100095</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>Josh Morrisey</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>ML100095_JOSH_MORRISEY_amzasset1.jpg</t>
+        </is>
+      </c>
+      <c r="D165" s="3" t="inlineStr">
+        <is>
+          <t>https://images-production-a1f5.up.railway.app/amz/asset-1/ML100095_JOSH_MORRISEY_amzasset1.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>ML100141</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>Alex Ovechkin Special Edition</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>ML100141_ALEX_OVECHKIN_SPECIAL_EDITION_amzasset1.jpg</t>
+        </is>
+      </c>
+      <c r="D166" s="3" t="inlineStr">
+        <is>
+          <t>https://images-production-a1f5.up.railway.app/amz/asset-1/ML100141_ALEX_OVECHKIN_SPECIAL_EDITION_amzasset1.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>ML100151</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>Pat Quinn Bench Boss Edition</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>ML100151_PAT_QUINN_BENCH_BOSS_EDITION_amzasset1.jpg</t>
+        </is>
+      </c>
+      <c r="D167" s="3" t="inlineStr">
+        <is>
+          <t>https://images-production-a1f5.up.railway.app/amz/asset-1/ML100151_PAT_QUINN_BENCH_BOSS_EDITION_amzasset1.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>ML100154</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>Matthew Schaefer</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>ML100154_MATTHEW_SCHAEFER_amzasset1.jpg</t>
+        </is>
+      </c>
+      <c r="D168" s="3" t="inlineStr">
+        <is>
+          <t>https://images-production-a1f5.up.railway.app/amz/asset-1/ML100154_MATTHEW_SCHAEFER_amzasset1.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>ML101193</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>Ivan Demidov Away</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>ML101193_IVAN_DEMIDOV_AWAY_amzasset1.jpg</t>
+        </is>
+      </c>
+      <c r="D169" s="3" t="inlineStr">
+        <is>
+          <t>https://images-production-a1f5.up.railway.app/amz/asset-1/ML101193_IVAN_DEMIDOV_AWAY_amzasset1.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>ML101212</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>Gavin Mckenna 2</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>ML101212_GAVIN_MCKENNA_2_amzasset1.jpg</t>
+        </is>
+      </c>
+      <c r="D170" s="3" t="inlineStr">
+        <is>
+          <t>https://images-production-a1f5.up.railway.app/amz/asset-1/ML101212_GAVIN_MCKENNA_2_amzasset1.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D164"/>
+  <autoFilter ref="A1:D170"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -4226,6 +4358,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D162" r:id="rId161"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D163" r:id="rId162"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D164" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D165" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D166" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D167" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D168" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D169" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D170" r:id="rId169"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>